<commit_message>
feat(auth): integrate premium Urban Jungle botanical login sanctuary matching reference design
</commit_message>
<xml_diff>
--- a/Flexi_Credit_Data.xlsx
+++ b/Flexi_Credit_Data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="107" uniqueCount="75">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="59">
   <si>
     <t>Order ID</t>
   </si>
@@ -74,72 +74,39 @@
     <t>Shipping Address</t>
   </si>
   <si>
-    <t>UJ-756866</t>
-  </si>
-  <si>
-    <t>2026-10-23 11:39:21</t>
-  </si>
-  <si>
-    <t>CUST-7113</t>
-  </si>
-  <si>
-    <t>Sameer Kardbhajne</t>
-  </si>
-  <si>
-    <t>sameer.kardbhajne@example.com</t>
-  </si>
-  <si>
-    <t>+1 (555) 379-6846</t>
+    <t>Email</t>
+  </si>
+  <si>
+    <t>Phone Number</t>
+  </si>
+  <si>
+    <t>Registration Date</t>
+  </si>
+  <si>
+    <t>Total Number of Orders</t>
+  </si>
+  <si>
+    <t>Total Amount Spent</t>
+  </si>
+  <si>
+    <t>Most Recent Order Date</t>
+  </si>
+  <si>
+    <t>Scientific Name</t>
+  </si>
+  <si>
+    <t>Category</t>
+  </si>
+  <si>
+    <t>Available Stock</t>
+  </si>
+  <si>
+    <t>Product Status</t>
   </si>
   <si>
     <t>Monstera Deliciosa</t>
   </si>
   <si>
-    <t>Credit Card</t>
-  </si>
-  <si>
-    <t>Paid</t>
-  </si>
-  <si>
-    <t>Confirmed</t>
-  </si>
-  <si>
-    <t>Shiv Sai Nagar Nagpur, Nagpur 441204</t>
-  </si>
-  <si>
-    <t>Email</t>
-  </si>
-  <si>
-    <t>Phone Number</t>
-  </si>
-  <si>
-    <t>Registration Date</t>
-  </si>
-  <si>
-    <t>Total Number of Orders</t>
-  </si>
-  <si>
-    <t>Total Amount Spent</t>
-  </si>
-  <si>
-    <t>Most Recent Order Date</t>
-  </si>
-  <si>
-    <t>2026-10-23</t>
-  </si>
-  <si>
-    <t>Scientific Name</t>
-  </si>
-  <si>
-    <t>Category</t>
-  </si>
-  <si>
-    <t>Available Stock</t>
-  </si>
-  <si>
-    <t>Product Status</t>
-  </si>
-  <si>
     <t>Monstera deliciosa</t>
   </si>
   <si>
@@ -215,12 +182,6 @@
     <t>Transaction Reference</t>
   </si>
   <si>
-    <t>PAY-756866</t>
-  </si>
-  <si>
-    <t>TXN-56923244</t>
-  </si>
-  <si>
     <t>Previous Status</t>
   </si>
   <si>
@@ -231,15 +192,6 @@
   </si>
   <si>
     <t>Updated By</t>
-  </si>
-  <si>
-    <t>Created</t>
-  </si>
-  <si>
-    <t>2026-10-23 11:39:11</t>
-  </si>
-  <si>
-    <t>System / Customer Checkout</t>
   </si>
 </sst>
 </file>
@@ -669,7 +621,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S2"/>
+  <dimension ref="A1:S1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -749,65 +701,6 @@
         <v>18</v>
       </c>
     </row>
-    <row r="2" ht="20" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="F2" s="4" t="s">
-        <v>24</v>
-      </c>
-      <c r="G2" s="4">
-        <v>1</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>25</v>
-      </c>
-      <c r="I2" s="4">
-        <v>1</v>
-      </c>
-      <c r="J2" s="5">
-        <v>45</v>
-      </c>
-      <c r="K2" s="5">
-        <v>45</v>
-      </c>
-      <c r="L2" s="5">
-        <v>0</v>
-      </c>
-      <c r="M2" s="5">
-        <v>0</v>
-      </c>
-      <c r="N2" s="5">
-        <v>0</v>
-      </c>
-      <c r="O2" s="5">
-        <v>45</v>
-      </c>
-      <c r="P2" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="Q2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="R2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="S2" s="4" t="s">
-        <v>29</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -817,7 +710,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -837,48 +730,22 @@
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>30</v>
+        <v>19</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>31</v>
+        <v>20</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>32</v>
+        <v>21</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>33</v>
+        <v>22</v>
       </c>
       <c r="G1" s="3" t="s">
-        <v>34</v>
+        <v>23</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>35</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>22</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D2" s="4" t="s">
         <v>24</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" s="4">
-        <v>1</v>
-      </c>
-      <c r="G2" s="5">
-        <v>45</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>20</v>
       </c>
     </row>
   </sheetData>
@@ -908,19 +775,19 @@
         <v>7</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>38</v>
+        <v>26</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>39</v>
+        <v>27</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -928,13 +795,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>41</v>
+        <v>30</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="E2" s="5">
         <v>45</v>
@@ -943,7 +810,7 @@
         <v>50</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -951,13 +818,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>44</v>
+        <v>33</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>45</v>
+        <v>34</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E3" s="7">
         <v>65</v>
@@ -966,7 +833,7 @@
         <v>50</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -974,13 +841,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>47</v>
+        <v>36</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>48</v>
+        <v>37</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E4" s="5">
         <v>30</v>
@@ -989,7 +856,7 @@
         <v>50</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -997,13 +864,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>50</v>
+        <v>39</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>51</v>
+        <v>40</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E5" s="7">
         <v>25</v>
@@ -1012,7 +879,7 @@
         <v>50</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1020,13 +887,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>52</v>
+        <v>41</v>
       </c>
       <c r="E6" s="5">
         <v>85</v>
@@ -1035,7 +902,7 @@
         <v>50</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1043,13 +910,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>55</v>
+        <v>44</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>56</v>
+        <v>45</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>57</v>
+        <v>46</v>
       </c>
       <c r="E7" s="7">
         <v>38</v>
@@ -1058,7 +925,7 @@
         <v>50</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1066,13 +933,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>58</v>
+        <v>47</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>59</v>
+        <v>48</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>49</v>
+        <v>38</v>
       </c>
       <c r="E8" s="5">
         <v>32</v>
@@ -1081,7 +948,7 @@
         <v>50</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -1089,13 +956,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>60</v>
+        <v>49</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>46</v>
+        <v>35</v>
       </c>
       <c r="E9" s="7">
         <v>55</v>
@@ -1104,7 +971,7 @@
         <v>50</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>
@@ -1116,7 +983,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H2"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -1129,7 +996,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>62</v>
+        <v>51</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1138,42 +1005,19 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>63</v>
+        <v>52</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>64</v>
+        <v>53</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>65</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>66</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>21</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>20</v>
-      </c>
-      <c r="F2" s="5">
-        <v>45</v>
-      </c>
-      <c r="G2" s="4" t="s">
-        <v>27</v>
-      </c>
-      <c r="H2" s="4" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
     </row>
   </sheetData>
@@ -1185,7 +1029,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E2"/>
+  <dimension ref="A1:E1"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1199,33 +1043,16 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>69</v>
+        <v>56</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>71</v>
-      </c>
-    </row>
-    <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="4" t="s">
-        <v>19</v>
-      </c>
-      <c r="B2" s="4" t="s">
-        <v>72</v>
-      </c>
-      <c r="C2" s="4" t="s">
-        <v>28</v>
-      </c>
-      <c r="D2" s="4" t="s">
-        <v>73</v>
-      </c>
-      <c r="E2" s="4" t="s">
-        <v>74</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
feat(backend): complete local MongoDB integration, customer sync, and submission documentation
</commit_message>
<xml_diff>
--- a/Flexi_Credit_Data.xlsx
+++ b/Flexi_Credit_Data.xlsx
@@ -15,7 +15,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="79" uniqueCount="59">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="84">
   <si>
     <t>Order ID</t>
   </si>
@@ -74,6 +74,63 @@
     <t>Shipping Address</t>
   </si>
   <si>
+    <t>UJ-822536</t>
+  </si>
+  <si>
+    <t>2026-10-26 12:53:17</t>
+  </si>
+  <si>
+    <t>CUST-7141</t>
+  </si>
+  <si>
+    <t>Alex Green</t>
+  </si>
+  <si>
+    <t>alex.green@urbanjungle.com</t>
+  </si>
+  <si>
+    <t>+1 555-432-1098</t>
+  </si>
+  <si>
+    <t>Snake Plant Laurentii</t>
+  </si>
+  <si>
+    <t>Credit Card</t>
+  </si>
+  <si>
+    <t>Paid</t>
+  </si>
+  <si>
+    <t>Confirmed</t>
+  </si>
+  <si>
+    <t>456 Botanical Rd, Pune 411038</t>
+  </si>
+  <si>
+    <t>UJ-650249</t>
+  </si>
+  <si>
+    <t>2026-10-26 12:49:32</t>
+  </si>
+  <si>
+    <t>CUST-7897</t>
+  </si>
+  <si>
+    <t>Sameer Karadbhajne</t>
+  </si>
+  <si>
+    <t>sameer.ca@urbanjungle.com</t>
+  </si>
+  <si>
+    <t>+1 (555) 498-5654</t>
+  </si>
+  <si>
+    <t>Monstera Deliciosa</t>
+  </si>
+  <si>
+    <t>123 College St, Pune 411001</t>
+  </si>
+  <si>
     <t>Email</t>
   </si>
   <si>
@@ -92,6 +149,9 @@
     <t>Most Recent Order Date</t>
   </si>
   <si>
+    <t>2026-10-26</t>
+  </si>
+  <si>
     <t>Scientific Name</t>
   </si>
   <si>
@@ -104,9 +164,6 @@
     <t>Product Status</t>
   </si>
   <si>
-    <t>Monstera Deliciosa</t>
-  </si>
-  <si>
     <t>Monstera deliciosa</t>
   </si>
   <si>
@@ -182,6 +239,18 @@
     <t>Transaction Reference</t>
   </si>
   <si>
+    <t>PAY-822536</t>
+  </si>
+  <si>
+    <t>TXN-92051118</t>
+  </si>
+  <si>
+    <t>PAY-650249</t>
+  </si>
+  <si>
+    <t>TXN-51358659</t>
+  </si>
+  <si>
     <t>Previous Status</t>
   </si>
   <si>
@@ -192,6 +261,12 @@
   </si>
   <si>
     <t>Updated By</t>
+  </si>
+  <si>
+    <t>Created</t>
+  </si>
+  <si>
+    <t>System / Customer Checkout</t>
   </si>
 </sst>
 </file>
@@ -621,7 +696,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:S3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -701,6 +776,124 @@
         <v>18</v>
       </c>
     </row>
+    <row r="2" ht="20" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="F2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="G2" s="4">
+        <v>2</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="I2" s="4">
+        <v>2</v>
+      </c>
+      <c r="J2" s="5">
+        <v>32</v>
+      </c>
+      <c r="K2" s="5">
+        <v>64</v>
+      </c>
+      <c r="L2" s="5">
+        <v>0</v>
+      </c>
+      <c r="M2" s="5">
+        <v>0</v>
+      </c>
+      <c r="N2" s="5">
+        <v>0</v>
+      </c>
+      <c r="O2" s="5">
+        <v>64</v>
+      </c>
+      <c r="P2" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="R2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="S2" s="4" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:19" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="F3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="G3" s="6">
+        <v>1</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>36</v>
+      </c>
+      <c r="I3" s="6">
+        <v>1</v>
+      </c>
+      <c r="J3" s="7">
+        <v>45</v>
+      </c>
+      <c r="K3" s="7">
+        <v>45</v>
+      </c>
+      <c r="L3" s="7">
+        <v>0</v>
+      </c>
+      <c r="M3" s="7">
+        <v>0</v>
+      </c>
+      <c r="N3" s="7">
+        <v>0</v>
+      </c>
+      <c r="O3" s="7">
+        <v>45</v>
+      </c>
+      <c r="P3" s="6" t="s">
+        <v>26</v>
+      </c>
+      <c r="Q3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="R3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="S3" s="6" t="s">
+        <v>37</v>
+      </c>
+    </row>
   </sheetData>
   <autoFilter ref="A1:S1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -710,7 +903,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -730,22 +923,74 @@
         <v>3</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>19</v>
+        <v>38</v>
       </c>
       <c r="D1" s="2" t="s">
+        <v>39</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>41</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>22</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>23</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>44</v>
+      </c>
+      <c r="F2" s="4">
+        <v>2</v>
+      </c>
+      <c r="G2" s="5">
+        <v>128</v>
+      </c>
+      <c r="H2" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E1" s="2" t="s">
-        <v>21</v>
-      </c>
-      <c r="F1" s="2" t="s">
-        <v>22</v>
-      </c>
-      <c r="G1" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="H1" s="2" t="s">
-        <v>24</v>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>33</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>44</v>
+      </c>
+      <c r="F3" s="6">
+        <v>1</v>
+      </c>
+      <c r="G3" s="7">
+        <v>45</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>31</v>
       </c>
     </row>
   </sheetData>
@@ -775,19 +1020,19 @@
         <v>7</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>25</v>
+        <v>45</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>26</v>
+        <v>46</v>
       </c>
       <c r="E1" s="3" t="s">
         <v>9</v>
       </c>
       <c r="F1" s="2" t="s">
-        <v>27</v>
+        <v>47</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>28</v>
+        <v>48</v>
       </c>
     </row>
     <row r="2" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -795,13 +1040,13 @@
         <v>1</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="C2" s="4" t="s">
-        <v>30</v>
+        <v>49</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>31</v>
+        <v>50</v>
       </c>
       <c r="E2" s="5">
         <v>45</v>
@@ -810,7 +1055,7 @@
         <v>50</v>
       </c>
       <c r="G2" s="4" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -818,13 +1063,13 @@
         <v>2</v>
       </c>
       <c r="B3" s="6" t="s">
-        <v>33</v>
+        <v>52</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>34</v>
+        <v>53</v>
       </c>
       <c r="D3" s="6" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="E3" s="7">
         <v>65</v>
@@ -833,7 +1078,7 @@
         <v>50</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -841,13 +1086,13 @@
         <v>3</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>36</v>
+        <v>55</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>37</v>
+        <v>56</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="E4" s="5">
         <v>30</v>
@@ -856,7 +1101,7 @@
         <v>50</v>
       </c>
       <c r="G4" s="4" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="5" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -864,13 +1109,13 @@
         <v>4</v>
       </c>
       <c r="B5" s="6" t="s">
-        <v>39</v>
+        <v>58</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>40</v>
+        <v>59</v>
       </c>
       <c r="D5" s="6" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="E5" s="7">
         <v>25</v>
@@ -879,7 +1124,7 @@
         <v>50</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -887,13 +1132,13 @@
         <v>5</v>
       </c>
       <c r="B6" s="4" t="s">
-        <v>42</v>
+        <v>61</v>
       </c>
       <c r="C6" s="4" t="s">
-        <v>43</v>
+        <v>62</v>
       </c>
       <c r="D6" s="4" t="s">
-        <v>41</v>
+        <v>60</v>
       </c>
       <c r="E6" s="5">
         <v>85</v>
@@ -902,7 +1147,7 @@
         <v>50</v>
       </c>
       <c r="G6" s="4" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="7" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -910,13 +1155,13 @@
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>44</v>
+        <v>63</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>45</v>
+        <v>64</v>
       </c>
       <c r="D7" s="6" t="s">
-        <v>46</v>
+        <v>65</v>
       </c>
       <c r="E7" s="7">
         <v>38</v>
@@ -925,7 +1170,7 @@
         <v>50</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="8" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -933,13 +1178,13 @@
         <v>7</v>
       </c>
       <c r="B8" s="4" t="s">
-        <v>47</v>
+        <v>66</v>
       </c>
       <c r="C8" s="4" t="s">
-        <v>48</v>
+        <v>67</v>
       </c>
       <c r="D8" s="4" t="s">
-        <v>38</v>
+        <v>57</v>
       </c>
       <c r="E8" s="5">
         <v>32</v>
@@ -948,7 +1193,7 @@
         <v>50</v>
       </c>
       <c r="G8" s="4" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
     <row r="9" ht="20" customHeight="1" spans="1:7" x14ac:dyDescent="0.25">
@@ -956,13 +1201,13 @@
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
-        <v>49</v>
+        <v>68</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>50</v>
+        <v>69</v>
       </c>
       <c r="D9" s="6" t="s">
-        <v>35</v>
+        <v>54</v>
       </c>
       <c r="E9" s="7">
         <v>55</v>
@@ -971,7 +1216,7 @@
         <v>50</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>32</v>
+        <v>51</v>
       </c>
     </row>
   </sheetData>
@@ -983,7 +1228,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:H3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="18" customWidth="1"/>
@@ -996,7 +1241,7 @@
   <sheetData>
     <row r="1" ht="28" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="2" t="s">
-        <v>51</v>
+        <v>70</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>0</v>
@@ -1005,19 +1250,65 @@
         <v>2</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>52</v>
+        <v>71</v>
       </c>
       <c r="E1" s="2" t="s">
         <v>15</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>53</v>
+        <v>72</v>
       </c>
       <c r="G1" s="2" t="s">
         <v>16</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>54</v>
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>74</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>21</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="F2" s="5">
+        <v>64</v>
+      </c>
+      <c r="G2" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="H2" s="4" t="s">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>76</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" s="7">
+        <v>45</v>
+      </c>
+      <c r="G3" s="6" t="s">
+        <v>27</v>
+      </c>
+      <c r="H3" s="6" t="s">
+        <v>77</v>
       </c>
     </row>
   </sheetData>
@@ -1029,7 +1320,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:E1"/>
+  <dimension ref="A1:E3"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="1" width="16" customWidth="1"/>
@@ -1043,16 +1334,50 @@
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
-        <v>55</v>
+        <v>78</v>
       </c>
       <c r="C1" s="2" t="s">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="D1" s="2" t="s">
-        <v>57</v>
+        <v>80</v>
       </c>
       <c r="E1" s="2" t="s">
-        <v>58</v>
+        <v>81</v>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>82</v>
+      </c>
+      <c r="C2" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E2" s="4" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="3" ht="20" customHeight="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="6" t="s">
+        <v>30</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>82</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>28</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>31</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>83</v>
       </c>
     </row>
   </sheetData>

</xml_diff>